<commit_message>
Using differenceInDays instead of generating array of days
</commit_message>
<xml_diff>
--- a/api/templates/sz_mtb_stats/en.xlsx
+++ b/api/templates/sz_mtb_stats/en.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25028"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DB5B1C-F138-43BC-AEFA-D8757B5BC6CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F1C8C7-66D0-4C83-903D-A9AD994F78EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="63">
   <si>
     <t>Monthly stats to be collated for GeneExpert</t>
   </si>
@@ -121,9 +121,6 @@
     <t>Average tests done per day</t>
   </si>
   <si>
-    <t>Mbabane central lab</t>
-  </si>
-  <si>
     <t>MTB +ve Trace</t>
   </si>
   <si>
@@ -215,6 +212,12 @@
   </si>
   <si>
     <t>total tests</t>
+  </si>
+  <si>
+    <t>&lt;Dates&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Sites&gt;</t>
   </si>
 </sst>
 </file>
@@ -533,32 +536,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -566,22 +585,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -944,225 +947,225 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="12">
-        <v>44562</v>
+        <v>62</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:9" s="11" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="30"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="36"/>
     </row>
     <row r="4" spans="1:9" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="26" t="s">
+      <c r="A8" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="32"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="21"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="26" t="s">
+      <c r="A9" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="26" t="s">
+      <c r="A13" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
       <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="18"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="29"/>
       <c r="G14" s="9"/>
       <c r="I14" s="13"/>
     </row>
     <row r="15" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="33"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="33"/>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
     </row>
     <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="34" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
+      <c r="A16" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
       <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A20" s="26" t="s">
+      <c r="A20" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="26"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="27"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="20"/>
       <c r="L20" s="14"/>
       <c r="M20" s="14"/>
       <c r="N20" s="14"/>
       <c r="O20" s="14"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A21" s="26" t="s">
+      <c r="A21" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
       <c r="G21" s="10"/>
       <c r="L21" s="14"/>
       <c r="M21" s="14"/>
@@ -1170,14 +1173,14 @@
       <c r="O21" s="14"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A22" s="26" t="s">
+      <c r="A22" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
       <c r="G22" s="1"/>
       <c r="L22" s="14"/>
       <c r="M22" s="15"/>
@@ -1197,14 +1200,14 @@
       <c r="O24" s="14"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="21"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="32"/>
       <c r="G25" s="13"/>
     </row>
     <row r="26" spans="1:15" ht="28.5" x14ac:dyDescent="0.2">
@@ -1221,7 +1224,7 @@
         <v>23</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>24</v>
@@ -1238,12 +1241,12 @@
       <c r="G27" s="13"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="F28" s="22"/>
+      <c r="F28" s="16"/>
       <c r="G28" s="13"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B29">
         <v>2</v>
@@ -1251,71 +1254,77 @@
       <c r="G29" s="13"/>
     </row>
     <row r="30" spans="1:15" ht="18" x14ac:dyDescent="0.25">
-      <c r="A30" s="35" t="s">
+      <c r="A30" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="36"/>
-      <c r="C30" s="36"/>
-      <c r="D30" s="36"/>
-      <c r="E30" s="36"/>
-      <c r="F30" s="36"/>
-      <c r="G30" s="36"/>
-      <c r="H30" s="36"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="23"/>
     </row>
     <row r="31" spans="1:15" ht="15" x14ac:dyDescent="0.25">
-      <c r="A31" s="25" t="s">
+      <c r="A31" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="D31" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="E31" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="H31" s="19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A32" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="D31" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="E31" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="F31" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="G31" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="H31" s="25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A32" s="23" t="s">
+      <c r="C32" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="F32" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="G32" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="B32" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C32" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="D32" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="E32" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="F32" s="23" t="s">
+      <c r="H32" s="18" t="s">
         <v>51</v>
-      </c>
-      <c r="G32" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="H32" s="24" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A7:F7"/>
     <mergeCell ref="A30:H30"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A22:F22"/>
@@ -1332,12 +1341,6 @@
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <conditionalFormatting sqref="G14">
     <cfRule type="cellIs" dxfId="0" priority="4" operator="greaterThan">
@@ -1356,67 +1359,67 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1432,22 +1435,22 @@
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>